<commit_message>
Fixed : Import School
</commit_message>
<xml_diff>
--- a/_Page/Sekolah/Template-Sekolah.xlsx
+++ b/_Page/Sekolah/Template-Sekolah.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RTG\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp64\www\rtgadd\_Page\Sekolah\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{16BB7919-B105-4121-A4E1-D463D60373EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09BB8133-7469-4DBB-B0BD-49A3D4BA23FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{957FBDA5-56DF-473A-92F3-6209DACFDE50}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="26">
   <si>
     <t>NPSN</t>
   </si>
@@ -56,52 +56,64 @@
     <t>MUARO JAMBI</t>
   </si>
   <si>
-    <t>10503561</t>
-  </si>
-  <si>
-    <t>SMP NEGERI 37 MUARA JAMBI</t>
-  </si>
-  <si>
-    <t>10503022</t>
-  </si>
-  <si>
-    <t>SD NEGERI 018/IX RENGAS BANDUNG</t>
-  </si>
-  <si>
-    <t>10502753</t>
-  </si>
-  <si>
-    <t>SD NEGERI 112IX MARO SEBO</t>
-  </si>
-  <si>
-    <t>10503014</t>
-  </si>
-  <si>
-    <t>SD NEGERI 022/IX TANGKIT</t>
-  </si>
-  <si>
-    <t>69888571</t>
-  </si>
-  <si>
-    <t>SD NEGERI 244/IX KEBUN SAYUR</t>
-  </si>
-  <si>
-    <t>10502825</t>
-  </si>
-  <si>
-    <t>SMP NEGERI 8 MUARO JAMBI</t>
-  </si>
-  <si>
-    <t>Kode Provinsi</t>
-  </si>
-  <si>
     <t>Nama Provinsi</t>
   </si>
   <si>
-    <t>Kode Kabupaten/Kota</t>
-  </si>
-  <si>
     <t>Nama Kabupaten</t>
+  </si>
+  <si>
+    <t>Kode Provinsi (BPS)</t>
+  </si>
+  <si>
+    <t>Kode Provinsi (DAPODIK)</t>
+  </si>
+  <si>
+    <t>Kode Kabupaten/Kota (BPS)</t>
+  </si>
+  <si>
+    <t>Kode Kabupaten/Kota (DAPODIK)</t>
+  </si>
+  <si>
+    <t>100000</t>
+  </si>
+  <si>
+    <t>100700</t>
+  </si>
+  <si>
+    <t>69859483</t>
+  </si>
+  <si>
+    <t>TK NEGERI 29 PULAU MENTARO</t>
+  </si>
+  <si>
+    <t>10507316</t>
+  </si>
+  <si>
+    <t>SMP NEGERI 44 MUARO JAMBI</t>
+  </si>
+  <si>
+    <t>10502785</t>
+  </si>
+  <si>
+    <t>SMP NEGERI 40 MUARO JAMBI</t>
+  </si>
+  <si>
+    <t>10503007</t>
+  </si>
+  <si>
+    <t>SD NEGERI 032IX SUKA DAMAI</t>
+  </si>
+  <si>
+    <t>10502810</t>
+  </si>
+  <si>
+    <t>SMP NEGERI 21 MUARO JAMBI</t>
+  </si>
+  <si>
+    <t>10502813</t>
+  </si>
+  <si>
+    <t>SMP NEGERI 24 MUARO JAMBI</t>
   </si>
 </sst>
 </file>
@@ -482,155 +494,199 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF50B76F-F402-46E9-A614-E380FDB9736B}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="33.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F2" t="s">
-        <v>7</v>
+      <c r="G2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" t="s">
+        <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>4</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
         <v>5</v>
       </c>
-      <c r="E3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
+      <c r="G3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" t="s">
         <v>5</v>
       </c>
-      <c r="E4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" t="s">
-        <v>11</v>
+      <c r="G4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H4" t="s">
+        <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
       <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
         <v>3</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>4</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" t="s">
         <v>5</v>
       </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" t="s">
-        <v>13</v>
+      <c r="G5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" t="s">
+        <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>2</v>
       </c>
       <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
         <v>3</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>4</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" t="s">
         <v>5</v>
       </c>
-      <c r="E6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" t="s">
-        <v>15</v>
+      <c r="G6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" t="s">
+        <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>2</v>
       </c>
       <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
         <v>3</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>4</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" t="s">
         <v>5</v>
       </c>
-      <c r="E7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7" t="s">
-        <v>17</v>
+      <c r="G7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>